<commit_message>
cambiuos en generaicon de iaas, checvar en produccion la grafica de iaas
</commit_message>
<xml_diff>
--- a/Data/INDICADORES/IAAS/2026/IAAS_2026.xlsx
+++ b/Data/INDICADORES/IAAS/2026/IAAS_2026.xlsx
@@ -7,12 +7,12 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="IASS 01" sheetId="1" r:id="rId1"/>
-    <sheet name="IASS 02" sheetId="2" r:id="rId2"/>
-    <sheet name="IASS 03" sheetId="3" r:id="rId3"/>
-    <sheet name="IASS 04" sheetId="4" r:id="rId4"/>
-    <sheet name="IASS 05" sheetId="5" r:id="rId5"/>
-    <sheet name="IASS 06" sheetId="6" r:id="rId6"/>
+    <sheet name="IAAS 01" sheetId="1" r:id="rId1"/>
+    <sheet name="IAAS 02" sheetId="2" r:id="rId2"/>
+    <sheet name="IAAS 03" sheetId="3" r:id="rId3"/>
+    <sheet name="IAAS 04" sheetId="4" r:id="rId4"/>
+    <sheet name="IAAS 05" sheetId="5" r:id="rId5"/>
+    <sheet name="IAAS 06" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -42,7 +42,7 @@
     <t>HGSMF 7 SAN FCO. DEL R.</t>
   </si>
   <si>
-    <t>HGSZ 10 GUANAJUATO</t>
+    <t>HGS 10 GUANAJUATO</t>
   </si>
   <si>
     <t>HGSMF 20 SAN LUIS DE</t>
@@ -1052,9 +1052,15 @@
         <v>6.81</v>
       </c>
       <c r="V7" s="6"/>
-      <c r="W7" s="6"/>
-      <c r="X7" s="6"/>
-      <c r="Y7" s="6"/>
+      <c r="W7" s="6">
+        <v>6</v>
+      </c>
+      <c r="X7" s="6">
+        <v>881</v>
+      </c>
+      <c r="Y7" s="7">
+        <v>6.81</v>
+      </c>
       <c r="AB7" s="6"/>
       <c r="AC7" s="6">
         <v>11</v>
@@ -1096,9 +1102,15 @@
         <v>5.92</v>
       </c>
       <c r="AR7" s="6"/>
-      <c r="AS7" s="6"/>
-      <c r="AT7" s="6"/>
-      <c r="AU7" s="6"/>
+      <c r="AS7" s="6">
+        <v>33</v>
+      </c>
+      <c r="AT7" s="6">
+        <v>5440</v>
+      </c>
+      <c r="AU7" s="7">
+        <v>6.07</v>
+      </c>
     </row>
     <row r="8" spans="1:47" ht="20" customHeight="1">
       <c r="A8" s="5" t="s">
@@ -1155,9 +1167,15 @@
         <v>4.41</v>
       </c>
       <c r="V8" s="10"/>
-      <c r="W8" s="10"/>
-      <c r="X8" s="10"/>
-      <c r="Y8" s="10"/>
+      <c r="W8" s="10">
+        <v>21</v>
+      </c>
+      <c r="X8" s="10">
+        <v>4759</v>
+      </c>
+      <c r="Y8" s="9">
+        <v>4.41</v>
+      </c>
       <c r="AB8" s="10"/>
       <c r="AC8" s="10">
         <v>48</v>
@@ -1199,9 +1217,15 @@
         <v>4.27</v>
       </c>
       <c r="AR8" s="10"/>
-      <c r="AS8" s="10"/>
-      <c r="AT8" s="10"/>
-      <c r="AU8" s="10"/>
+      <c r="AS8" s="10">
+        <v>126</v>
+      </c>
+      <c r="AT8" s="10">
+        <v>29334</v>
+      </c>
+      <c r="AU8" s="9">
+        <v>4.3</v>
+      </c>
     </row>
     <row r="9" spans="1:47" ht="20" customHeight="1">
       <c r="A9" s="5" t="s">
@@ -1258,9 +1282,15 @@
         <v>0</v>
       </c>
       <c r="V9" s="6"/>
-      <c r="W9" s="6"/>
-      <c r="X9" s="6"/>
-      <c r="Y9" s="6"/>
+      <c r="W9" s="6">
+        <v>0</v>
+      </c>
+      <c r="X9" s="6">
+        <v>378</v>
+      </c>
+      <c r="Y9" s="8">
+        <v>0</v>
+      </c>
       <c r="AB9" s="6"/>
       <c r="AC9" s="6">
         <v>0</v>
@@ -1302,112 +1332,76 @@
         <v>0</v>
       </c>
       <c r="AR9" s="6"/>
-      <c r="AS9" s="6"/>
-      <c r="AT9" s="6"/>
-      <c r="AU9" s="6"/>
+      <c r="AS9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AT9" s="6">
+        <v>2454</v>
+      </c>
+      <c r="AU9" s="8">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:47" ht="20" customHeight="1">
       <c r="A10" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="10"/>
-      <c r="C10" s="10">
-        <v>2</v>
-      </c>
-      <c r="D10" s="10">
-        <v>704</v>
-      </c>
-      <c r="E10" s="9">
-        <v>2.84</v>
-      </c>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
       <c r="F10" s="10"/>
-      <c r="G10" s="10">
-        <v>5</v>
-      </c>
-      <c r="H10" s="10">
-        <v>687</v>
-      </c>
-      <c r="I10" s="8">
-        <v>7.27</v>
-      </c>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
       <c r="J10" s="10"/>
-      <c r="K10" s="10">
-        <v>3</v>
-      </c>
-      <c r="L10" s="10">
-        <v>631</v>
-      </c>
-      <c r="M10" s="7">
-        <v>4.75</v>
-      </c>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
       <c r="N10" s="10"/>
-      <c r="O10" s="10">
-        <v>5</v>
-      </c>
-      <c r="P10" s="10">
-        <v>699</v>
-      </c>
-      <c r="Q10" s="8">
-        <v>7.15</v>
-      </c>
+      <c r="O10" s="10"/>
+      <c r="P10" s="10"/>
+      <c r="Q10" s="10"/>
       <c r="R10" s="10"/>
-      <c r="S10" s="10">
-        <v>5</v>
-      </c>
-      <c r="T10" s="10">
+      <c r="S10" s="10"/>
+      <c r="T10" s="10"/>
+      <c r="U10" s="10"/>
+      <c r="V10" s="10"/>
+      <c r="W10" s="10">
+        <v>0</v>
+      </c>
+      <c r="X10" s="10">
         <v>658</v>
       </c>
-      <c r="U10" s="8">
-        <v>7.6</v>
-      </c>
-      <c r="V10" s="10"/>
-      <c r="W10" s="10"/>
-      <c r="X10" s="10"/>
-      <c r="Y10" s="10"/>
+      <c r="Y10" s="8">
+        <v>0</v>
+      </c>
       <c r="AB10" s="10"/>
-      <c r="AC10" s="10">
-        <v>7</v>
-      </c>
-      <c r="AD10" s="10">
-        <v>1391</v>
-      </c>
-      <c r="AE10" s="7">
-        <v>5.03</v>
-      </c>
+      <c r="AC10" s="10"/>
+      <c r="AD10" s="10"/>
+      <c r="AE10" s="10"/>
       <c r="AF10" s="10"/>
-      <c r="AG10" s="10">
-        <v>10</v>
-      </c>
-      <c r="AH10" s="10">
-        <v>2022</v>
-      </c>
-      <c r="AI10" s="7">
-        <v>4.95</v>
-      </c>
+      <c r="AG10" s="10"/>
+      <c r="AH10" s="10"/>
+      <c r="AI10" s="10"/>
       <c r="AJ10" s="10"/>
-      <c r="AK10" s="10">
-        <v>15</v>
-      </c>
-      <c r="AL10" s="10">
-        <v>2721</v>
-      </c>
-      <c r="AM10" s="7">
-        <v>5.51</v>
-      </c>
+      <c r="AK10" s="10"/>
+      <c r="AL10" s="10"/>
+      <c r="AM10" s="10"/>
       <c r="AN10" s="10"/>
-      <c r="AO10" s="10">
-        <v>20</v>
-      </c>
-      <c r="AP10" s="10">
-        <v>3379</v>
-      </c>
-      <c r="AQ10" s="7">
-        <v>5.92</v>
-      </c>
+      <c r="AO10" s="10"/>
+      <c r="AP10" s="10"/>
+      <c r="AQ10" s="10"/>
       <c r="AR10" s="10"/>
-      <c r="AS10" s="10"/>
-      <c r="AT10" s="10"/>
-      <c r="AU10" s="10"/>
+      <c r="AS10" s="10">
+        <v>0</v>
+      </c>
+      <c r="AT10" s="10">
+        <v>658</v>
+      </c>
+      <c r="AU10" s="8">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:47" ht="20" customHeight="1">
       <c r="A11" s="5" t="s">
@@ -1464,9 +1458,15 @@
         <v>0</v>
       </c>
       <c r="V11" s="6"/>
-      <c r="W11" s="6"/>
-      <c r="X11" s="6"/>
-      <c r="Y11" s="6"/>
+      <c r="W11" s="6">
+        <v>0</v>
+      </c>
+      <c r="X11" s="6">
+        <v>392</v>
+      </c>
+      <c r="Y11" s="8">
+        <v>0</v>
+      </c>
       <c r="AB11" s="6"/>
       <c r="AC11" s="6">
         <v>0</v>
@@ -1508,9 +1508,15 @@
         <v>0</v>
       </c>
       <c r="AR11" s="6"/>
-      <c r="AS11" s="6"/>
-      <c r="AT11" s="6"/>
-      <c r="AU11" s="6"/>
+      <c r="AS11" s="6">
+        <v>0</v>
+      </c>
+      <c r="AT11" s="6">
+        <v>1997</v>
+      </c>
+      <c r="AU11" s="8">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:47" ht="20" customHeight="1">
       <c r="A12" s="5" t="s">
@@ -1567,9 +1573,15 @@
         <v>16.73</v>
       </c>
       <c r="V12" s="10"/>
-      <c r="W12" s="10"/>
-      <c r="X12" s="10"/>
-      <c r="Y12" s="10"/>
+      <c r="W12" s="10">
+        <v>51</v>
+      </c>
+      <c r="X12" s="10">
+        <v>3049</v>
+      </c>
+      <c r="Y12" s="8">
+        <v>16.73</v>
+      </c>
       <c r="AB12" s="10"/>
       <c r="AC12" s="10">
         <v>134</v>
@@ -1611,9 +1623,15 @@
         <v>18.59</v>
       </c>
       <c r="AR12" s="10"/>
-      <c r="AS12" s="10"/>
-      <c r="AT12" s="10"/>
-      <c r="AU12" s="10"/>
+      <c r="AS12" s="10">
+        <v>338</v>
+      </c>
+      <c r="AT12" s="10">
+        <v>18485</v>
+      </c>
+      <c r="AU12" s="8">
+        <v>18.29</v>
+      </c>
     </row>
     <row r="13" spans="1:47" ht="20" customHeight="1">
       <c r="A13" s="5" t="s">
@@ -1670,9 +1688,15 @@
         <v>10.22</v>
       </c>
       <c r="V13" s="6"/>
-      <c r="W13" s="6"/>
-      <c r="X13" s="6"/>
-      <c r="Y13" s="6"/>
+      <c r="W13" s="6">
+        <v>20</v>
+      </c>
+      <c r="X13" s="6">
+        <v>1957</v>
+      </c>
+      <c r="Y13" s="7">
+        <v>10.22</v>
+      </c>
       <c r="AB13" s="6"/>
       <c r="AC13" s="6">
         <v>23</v>
@@ -1714,9 +1738,15 @@
         <v>6.99</v>
       </c>
       <c r="AR13" s="6"/>
-      <c r="AS13" s="6"/>
-      <c r="AT13" s="6"/>
-      <c r="AU13" s="6"/>
+      <c r="AS13" s="6">
+        <v>89</v>
+      </c>
+      <c r="AT13" s="6">
+        <v>11823</v>
+      </c>
+      <c r="AU13" s="7">
+        <v>7.53</v>
+      </c>
     </row>
     <row r="14" spans="1:47" ht="20" customHeight="1">
       <c r="A14" s="5" t="s">
@@ -1773,9 +1803,15 @@
         <v>0</v>
       </c>
       <c r="V14" s="10"/>
-      <c r="W14" s="10"/>
-      <c r="X14" s="10"/>
-      <c r="Y14" s="10"/>
+      <c r="W14" s="10">
+        <v>0</v>
+      </c>
+      <c r="X14" s="10">
+        <v>264</v>
+      </c>
+      <c r="Y14" s="8">
+        <v>0</v>
+      </c>
       <c r="AB14" s="10"/>
       <c r="AC14" s="10">
         <v>0</v>
@@ -1817,9 +1853,15 @@
         <v>0</v>
       </c>
       <c r="AR14" s="10"/>
-      <c r="AS14" s="10"/>
-      <c r="AT14" s="10"/>
-      <c r="AU14" s="10"/>
+      <c r="AS14" s="10">
+        <v>0</v>
+      </c>
+      <c r="AT14" s="10">
+        <v>1477</v>
+      </c>
+      <c r="AU14" s="8">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:47" ht="20" customHeight="1">
       <c r="A15" s="5" t="s">
@@ -1876,9 +1918,15 @@
         <v>10.69</v>
       </c>
       <c r="V15" s="6"/>
-      <c r="W15" s="6"/>
-      <c r="X15" s="6"/>
-      <c r="Y15" s="6"/>
+      <c r="W15" s="6">
+        <v>52</v>
+      </c>
+      <c r="X15" s="6">
+        <v>4863</v>
+      </c>
+      <c r="Y15" s="7">
+        <v>10.69</v>
+      </c>
       <c r="AB15" s="6"/>
       <c r="AC15" s="6">
         <v>88</v>
@@ -1920,9 +1968,15 @@
         <v>10.87</v>
       </c>
       <c r="AR15" s="6"/>
-      <c r="AS15" s="6"/>
-      <c r="AT15" s="6"/>
-      <c r="AU15" s="6"/>
+      <c r="AS15" s="6">
+        <v>321</v>
+      </c>
+      <c r="AT15" s="6">
+        <v>29618</v>
+      </c>
+      <c r="AU15" s="7">
+        <v>10.84</v>
+      </c>
     </row>
     <row r="16" spans="1:47" ht="20" customHeight="1">
       <c r="A16" s="5" t="s">
@@ -1979,9 +2033,15 @@
         <v>0</v>
       </c>
       <c r="V16" s="10"/>
-      <c r="W16" s="10"/>
-      <c r="X16" s="10"/>
-      <c r="Y16" s="10"/>
+      <c r="W16" s="10">
+        <v>0</v>
+      </c>
+      <c r="X16" s="10">
+        <v>308</v>
+      </c>
+      <c r="Y16" s="8">
+        <v>0</v>
+      </c>
       <c r="AB16" s="10"/>
       <c r="AC16" s="10">
         <v>0</v>
@@ -2023,9 +2083,15 @@
         <v>0</v>
       </c>
       <c r="AR16" s="10"/>
-      <c r="AS16" s="10"/>
-      <c r="AT16" s="10"/>
-      <c r="AU16" s="10"/>
+      <c r="AS16" s="10">
+        <v>0</v>
+      </c>
+      <c r="AT16" s="10">
+        <v>1994</v>
+      </c>
+      <c r="AU16" s="8">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="1:51" ht="20" customHeight="1">
       <c r="A17" s="5" t="s">
@@ -2082,9 +2148,15 @@
         <v>6.86</v>
       </c>
       <c r="V17" s="6"/>
-      <c r="W17" s="6"/>
-      <c r="X17" s="6"/>
-      <c r="Y17" s="6"/>
+      <c r="W17" s="6">
+        <v>51</v>
+      </c>
+      <c r="X17" s="6">
+        <v>7430</v>
+      </c>
+      <c r="Y17" s="9">
+        <v>6.86</v>
+      </c>
       <c r="AB17" s="6"/>
       <c r="AC17" s="6">
         <v>97</v>
@@ -2126,9 +2198,15 @@
         <v>7.48</v>
       </c>
       <c r="AR17" s="6"/>
-      <c r="AS17" s="6"/>
-      <c r="AT17" s="6"/>
-      <c r="AU17" s="6"/>
+      <c r="AS17" s="6">
+        <v>315</v>
+      </c>
+      <c r="AT17" s="6">
+        <v>42703</v>
+      </c>
+      <c r="AU17" s="7">
+        <v>7.38</v>
+      </c>
     </row>
     <row r="18" spans="1:51" ht="20" customHeight="1">
       <c r="A18" s="5" t="s">
@@ -2185,53 +2263,65 @@
         <v>8.26</v>
       </c>
       <c r="V18" s="11"/>
-      <c r="W18" s="11"/>
-      <c r="X18" s="11"/>
-      <c r="Y18" s="11"/>
+      <c r="W18" s="11">
+        <v>206</v>
+      </c>
+      <c r="X18" s="11">
+        <v>24939</v>
+      </c>
+      <c r="Y18" s="7">
+        <v>8.26</v>
+      </c>
       <c r="AB18" s="11"/>
       <c r="AC18" s="11">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="AD18" s="11">
-        <v>50497</v>
+        <v>49106</v>
       </c>
       <c r="AE18" s="7">
-        <v>8.08</v>
+        <v>8.17</v>
       </c>
       <c r="AF18" s="11"/>
       <c r="AG18" s="11">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="AH18" s="11">
-        <v>73608</v>
+        <v>71586</v>
       </c>
       <c r="AI18" s="7">
-        <v>8.44</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="AJ18" s="11"/>
       <c r="AK18" s="11">
-        <v>835</v>
+        <v>820</v>
       </c>
       <c r="AL18" s="11">
-        <v>99484</v>
+        <v>96763</v>
       </c>
       <c r="AM18" s="7">
-        <v>8.390000000000001</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="AN18" s="11"/>
       <c r="AO18" s="11">
-        <v>1041</v>
+        <v>1021</v>
       </c>
       <c r="AP18" s="11">
-        <v>124423</v>
+        <v>121044</v>
       </c>
       <c r="AQ18" s="7">
+        <v>8.43</v>
+      </c>
+      <c r="AR18" s="11"/>
+      <c r="AS18" s="11">
+        <v>1222</v>
+      </c>
+      <c r="AT18" s="11">
+        <v>145983</v>
+      </c>
+      <c r="AU18" s="7">
         <v>8.369999999999999</v>
       </c>
-      <c r="AR18" s="11"/>
-      <c r="AS18" s="11"/>
-      <c r="AT18" s="11"/>
-      <c r="AU18" s="11"/>
     </row>
     <row r="21" spans="1:51" ht="20" customHeight="1">
       <c r="A21" s="3" t="s">
@@ -3607,9 +3697,15 @@
       <c r="P5" s="7">
         <v>2.47</v>
       </c>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="6"/>
+      <c r="Q5" s="6">
+        <v>9</v>
+      </c>
+      <c r="R5" s="6">
+        <v>365</v>
+      </c>
+      <c r="S5" s="7">
+        <v>2.47</v>
+      </c>
       <c r="T5" s="6"/>
       <c r="U5" s="6"/>
       <c r="V5" s="6"/>
@@ -3678,9 +3774,15 @@
       <c r="P6" s="8">
         <v>0</v>
       </c>
-      <c r="Q6" s="10"/>
-      <c r="R6" s="10"/>
-      <c r="S6" s="10"/>
+      <c r="Q6" s="10">
+        <v>2</v>
+      </c>
+      <c r="R6" s="10">
+        <v>0</v>
+      </c>
+      <c r="S6" s="8">
+        <v>0</v>
+      </c>
       <c r="T6" s="10"/>
       <c r="U6" s="10"/>
       <c r="V6" s="10"/>
@@ -3749,9 +3851,15 @@
       <c r="P7" s="7">
         <v>2.18</v>
       </c>
-      <c r="Q7" s="6"/>
-      <c r="R7" s="6"/>
-      <c r="S7" s="6"/>
+      <c r="Q7" s="6">
+        <v>7</v>
+      </c>
+      <c r="R7" s="6">
+        <v>321</v>
+      </c>
+      <c r="S7" s="7">
+        <v>2.18</v>
+      </c>
       <c r="T7" s="6"/>
       <c r="U7" s="6"/>
       <c r="V7" s="6"/>
@@ -3776,37 +3884,37 @@
         <v>7</v>
       </c>
       <c r="B8" s="10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8" s="10">
-        <v>109</v>
+        <v>0</v>
       </c>
       <c r="D8" s="8">
-        <v>0.9174</v>
+        <v>0</v>
       </c>
       <c r="E8" s="10">
         <v>0</v>
       </c>
       <c r="F8" s="10">
-        <v>136</v>
+        <v>0</v>
       </c>
       <c r="G8" s="8">
         <v>0</v>
       </c>
       <c r="H8" s="10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="10">
-        <v>147</v>
+        <v>0</v>
       </c>
       <c r="J8" s="8">
-        <v>0.6803</v>
+        <v>0</v>
       </c>
       <c r="K8" s="10">
         <v>0</v>
       </c>
       <c r="L8" s="10">
-        <v>173</v>
+        <v>0</v>
       </c>
       <c r="M8" s="8">
         <v>0</v>
@@ -3815,14 +3923,20 @@
         <v>0</v>
       </c>
       <c r="O8" s="10">
-        <v>160</v>
+        <v>0</v>
       </c>
       <c r="P8" s="8">
         <v>0</v>
       </c>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="10"/>
-      <c r="S8" s="10"/>
+      <c r="Q8" s="10">
+        <v>0</v>
+      </c>
+      <c r="R8" s="10">
+        <v>0</v>
+      </c>
+      <c r="S8" s="8">
+        <v>0</v>
+      </c>
       <c r="T8" s="10"/>
       <c r="U8" s="10"/>
       <c r="V8" s="10"/>
@@ -3891,9 +4005,15 @@
       <c r="P9" s="8">
         <v>0</v>
       </c>
-      <c r="Q9" s="6"/>
-      <c r="R9" s="6"/>
-      <c r="S9" s="6"/>
+      <c r="Q9" s="6">
+        <v>0</v>
+      </c>
+      <c r="R9" s="6">
+        <v>0</v>
+      </c>
+      <c r="S9" s="8">
+        <v>0</v>
+      </c>
       <c r="T9" s="6"/>
       <c r="U9" s="6"/>
       <c r="V9" s="6"/>
@@ -3962,9 +4082,15 @@
       <c r="P10" s="7">
         <v>3.03</v>
       </c>
-      <c r="Q10" s="10"/>
-      <c r="R10" s="10"/>
-      <c r="S10" s="10"/>
+      <c r="Q10" s="10">
+        <v>8</v>
+      </c>
+      <c r="R10" s="10">
+        <v>264</v>
+      </c>
+      <c r="S10" s="7">
+        <v>3.03</v>
+      </c>
       <c r="T10" s="10"/>
       <c r="U10" s="10"/>
       <c r="V10" s="10"/>
@@ -4033,9 +4159,15 @@
       <c r="P11" s="7">
         <v>2.74</v>
       </c>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
+      <c r="Q11" s="6">
+        <v>2</v>
+      </c>
+      <c r="R11" s="6">
+        <v>73</v>
+      </c>
+      <c r="S11" s="7">
+        <v>2.74</v>
+      </c>
       <c r="T11" s="6"/>
       <c r="U11" s="6"/>
       <c r="V11" s="6"/>
@@ -4104,9 +4236,15 @@
       <c r="P12" s="8">
         <v>0</v>
       </c>
-      <c r="Q12" s="10"/>
-      <c r="R12" s="10"/>
-      <c r="S12" s="10"/>
+      <c r="Q12" s="10">
+        <v>13</v>
+      </c>
+      <c r="R12" s="10">
+        <v>0</v>
+      </c>
+      <c r="S12" s="8">
+        <v>0</v>
+      </c>
       <c r="T12" s="10"/>
       <c r="U12" s="10"/>
       <c r="V12" s="10"/>
@@ -4175,9 +4313,15 @@
       <c r="P13" s="8">
         <v>0</v>
       </c>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
-      <c r="S13" s="6"/>
+      <c r="Q13" s="6">
+        <v>0</v>
+      </c>
+      <c r="R13" s="6">
+        <v>0</v>
+      </c>
+      <c r="S13" s="8">
+        <v>0</v>
+      </c>
       <c r="T13" s="6"/>
       <c r="U13" s="6"/>
       <c r="V13" s="6"/>
@@ -4246,9 +4390,15 @@
       <c r="P14" s="8">
         <v>0</v>
       </c>
-      <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
-      <c r="S14" s="10"/>
+      <c r="Q14" s="10">
+        <v>0</v>
+      </c>
+      <c r="R14" s="10">
+        <v>0</v>
+      </c>
+      <c r="S14" s="8">
+        <v>0</v>
+      </c>
       <c r="T14" s="10"/>
       <c r="U14" s="10"/>
       <c r="V14" s="10"/>
@@ -4317,9 +4467,15 @@
       <c r="P15" s="8">
         <v>0</v>
       </c>
-      <c r="Q15" s="6"/>
-      <c r="R15" s="6"/>
-      <c r="S15" s="6"/>
+      <c r="Q15" s="6">
+        <v>0</v>
+      </c>
+      <c r="R15" s="6">
+        <v>0</v>
+      </c>
+      <c r="S15" s="8">
+        <v>0</v>
+      </c>
       <c r="T15" s="6"/>
       <c r="U15" s="6"/>
       <c r="V15" s="6"/>
@@ -4607,9 +4763,15 @@
       <c r="P20" s="7">
         <v>2.67</v>
       </c>
-      <c r="Q20" s="6"/>
-      <c r="R20" s="6"/>
-      <c r="S20" s="6"/>
+      <c r="Q20" s="6">
+        <v>54</v>
+      </c>
+      <c r="R20" s="6">
+        <v>2052</v>
+      </c>
+      <c r="S20" s="7">
+        <v>2.63</v>
+      </c>
       <c r="T20" s="6"/>
       <c r="U20" s="6"/>
       <c r="V20" s="6"/>
@@ -4678,9 +4840,15 @@
       <c r="P21" s="7">
         <v>2.1</v>
       </c>
-      <c r="Q21" s="10"/>
-      <c r="R21" s="10"/>
-      <c r="S21" s="10"/>
+      <c r="Q21" s="10">
+        <v>17</v>
+      </c>
+      <c r="R21" s="10">
+        <v>713</v>
+      </c>
+      <c r="S21" s="7">
+        <v>2.38</v>
+      </c>
       <c r="T21" s="10"/>
       <c r="U21" s="10"/>
       <c r="V21" s="10"/>
@@ -4749,9 +4917,15 @@
       <c r="P22" s="8">
         <v>4.06</v>
       </c>
-      <c r="Q22" s="6"/>
-      <c r="R22" s="6"/>
-      <c r="S22" s="6"/>
+      <c r="Q22" s="6">
+        <v>60</v>
+      </c>
+      <c r="R22" s="6">
+        <v>1625</v>
+      </c>
+      <c r="S22" s="8">
+        <v>3.69</v>
+      </c>
       <c r="T22" s="6"/>
       <c r="U22" s="6"/>
       <c r="V22" s="6"/>
@@ -4775,51 +4949,21 @@
       <c r="A23" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="10">
-        <v>1</v>
-      </c>
-      <c r="C23" s="10">
-        <v>109</v>
-      </c>
-      <c r="D23" s="8">
-        <v>0.92</v>
-      </c>
-      <c r="E23" s="10">
-        <v>1</v>
-      </c>
-      <c r="F23" s="10">
-        <v>245</v>
-      </c>
-      <c r="G23" s="8">
-        <v>0.41</v>
-      </c>
-      <c r="H23" s="10">
-        <v>2</v>
-      </c>
-      <c r="I23" s="10">
-        <v>392</v>
-      </c>
-      <c r="J23" s="8">
-        <v>0.51</v>
-      </c>
-      <c r="K23" s="10">
-        <v>2</v>
-      </c>
-      <c r="L23" s="10">
-        <v>565</v>
-      </c>
-      <c r="M23" s="8">
-        <v>0.35</v>
-      </c>
-      <c r="N23" s="10">
-        <v>2</v>
-      </c>
-      <c r="O23" s="10">
-        <v>725</v>
-      </c>
-      <c r="P23" s="8">
-        <v>0.28</v>
-      </c>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10"/>
       <c r="Q23" s="10"/>
       <c r="R23" s="10"/>
       <c r="S23" s="10"/>
@@ -4891,9 +5035,15 @@
       <c r="P24" s="8">
         <v>0</v>
       </c>
-      <c r="Q24" s="6"/>
-      <c r="R24" s="6"/>
-      <c r="S24" s="6"/>
+      <c r="Q24" s="6">
+        <v>0</v>
+      </c>
+      <c r="R24" s="6">
+        <v>0</v>
+      </c>
+      <c r="S24" s="8">
+        <v>0</v>
+      </c>
       <c r="T24" s="6"/>
       <c r="U24" s="6"/>
       <c r="V24" s="6"/>
@@ -4962,9 +5112,15 @@
       <c r="P25" s="7">
         <v>3.13</v>
       </c>
-      <c r="Q25" s="10"/>
-      <c r="R25" s="10"/>
-      <c r="S25" s="10"/>
+      <c r="Q25" s="10">
+        <v>50</v>
+      </c>
+      <c r="R25" s="10">
+        <v>1607</v>
+      </c>
+      <c r="S25" s="7">
+        <v>3.11</v>
+      </c>
       <c r="T25" s="10"/>
       <c r="U25" s="10"/>
       <c r="V25" s="10"/>
@@ -5033,9 +5189,15 @@
       <c r="P26" s="7">
         <v>2.31</v>
       </c>
-      <c r="Q26" s="6"/>
-      <c r="R26" s="6"/>
-      <c r="S26" s="6"/>
+      <c r="Q26" s="6">
+        <v>10</v>
+      </c>
+      <c r="R26" s="6">
+        <v>420</v>
+      </c>
+      <c r="S26" s="7">
+        <v>2.38</v>
+      </c>
       <c r="T26" s="6"/>
       <c r="U26" s="6"/>
       <c r="V26" s="6"/>
@@ -5104,9 +5266,15 @@
       <c r="P27" s="7">
         <v>2.43</v>
       </c>
-      <c r="Q27" s="10"/>
-      <c r="R27" s="10"/>
-      <c r="S27" s="10"/>
+      <c r="Q27" s="10">
+        <v>77</v>
+      </c>
+      <c r="R27" s="10">
+        <v>2637</v>
+      </c>
+      <c r="S27" s="7">
+        <v>2.92</v>
+      </c>
       <c r="T27" s="10"/>
       <c r="U27" s="10"/>
       <c r="V27" s="10"/>
@@ -5175,9 +5343,15 @@
       <c r="P28" s="8">
         <v>0</v>
       </c>
-      <c r="Q28" s="6"/>
-      <c r="R28" s="6"/>
-      <c r="S28" s="6"/>
+      <c r="Q28" s="6">
+        <v>0</v>
+      </c>
+      <c r="R28" s="6">
+        <v>0</v>
+      </c>
+      <c r="S28" s="8">
+        <v>0</v>
+      </c>
       <c r="T28" s="6"/>
       <c r="U28" s="6"/>
       <c r="V28" s="6"/>
@@ -5246,9 +5420,15 @@
       <c r="P29" s="8">
         <v>0</v>
       </c>
-      <c r="Q29" s="10"/>
-      <c r="R29" s="10"/>
-      <c r="S29" s="10"/>
+      <c r="Q29" s="10">
+        <v>0</v>
+      </c>
+      <c r="R29" s="10">
+        <v>0</v>
+      </c>
+      <c r="S29" s="8">
+        <v>0</v>
+      </c>
       <c r="T29" s="10"/>
       <c r="U29" s="10"/>
       <c r="V29" s="10"/>
@@ -5317,9 +5497,15 @@
       <c r="P30" s="8">
         <v>0</v>
       </c>
-      <c r="Q30" s="6"/>
-      <c r="R30" s="6"/>
-      <c r="S30" s="6"/>
+      <c r="Q30" s="6">
+        <v>0</v>
+      </c>
+      <c r="R30" s="6">
+        <v>0</v>
+      </c>
+      <c r="S30" s="8">
+        <v>0</v>
+      </c>
       <c r="T30" s="6"/>
       <c r="U30" s="6"/>
       <c r="V30" s="6"/>
@@ -5344,53 +5530,59 @@
         <v>15</v>
       </c>
       <c r="B31" s="11">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C31" s="11">
-        <v>1675</v>
+        <v>1566</v>
       </c>
       <c r="D31" s="7">
-        <v>2.15</v>
+        <v>2.23</v>
       </c>
       <c r="E31" s="11">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F31" s="11">
-        <v>3490</v>
+        <v>3245</v>
       </c>
       <c r="G31" s="7">
-        <v>2.92</v>
+        <v>3.11</v>
       </c>
       <c r="H31" s="11">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="I31" s="11">
-        <v>5329</v>
+        <v>4937</v>
       </c>
       <c r="J31" s="7">
-        <v>2.93</v>
+        <v>3.12</v>
       </c>
       <c r="K31" s="11">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="L31" s="11">
-        <v>7573</v>
+        <v>7008</v>
       </c>
       <c r="M31" s="7">
-        <v>2.48</v>
+        <v>2.65</v>
       </c>
       <c r="N31" s="11">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="O31" s="11">
-        <v>8756</v>
+        <v>8031</v>
       </c>
       <c r="P31" s="7">
-        <v>2.62</v>
-      </c>
-      <c r="Q31" s="11"/>
-      <c r="R31" s="11"/>
-      <c r="S31" s="11"/>
+        <v>2.83</v>
+      </c>
+      <c r="Q31" s="11">
+        <v>268</v>
+      </c>
+      <c r="R31" s="11">
+        <v>9054</v>
+      </c>
+      <c r="S31" s="7">
+        <v>2.96</v>
+      </c>
       <c r="T31" s="11"/>
       <c r="U31" s="11"/>
       <c r="V31" s="11"/>
@@ -5788,9 +5980,15 @@
       <c r="P5" s="8">
         <v>30.77</v>
       </c>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="6"/>
+      <c r="Q5" s="6">
+        <v>2</v>
+      </c>
+      <c r="R5" s="6">
+        <v>65</v>
+      </c>
+      <c r="S5" s="8">
+        <v>30.77</v>
+      </c>
       <c r="T5" s="6"/>
       <c r="U5" s="6"/>
       <c r="V5" s="6"/>
@@ -5859,9 +6057,15 @@
       <c r="P6" s="8">
         <v>0</v>
       </c>
-      <c r="Q6" s="10"/>
-      <c r="R6" s="10"/>
-      <c r="S6" s="10"/>
+      <c r="Q6" s="10">
+        <v>0</v>
+      </c>
+      <c r="R6" s="10">
+        <v>0</v>
+      </c>
+      <c r="S6" s="8">
+        <v>0</v>
+      </c>
       <c r="T6" s="10"/>
       <c r="U6" s="10"/>
       <c r="V6" s="10"/>
@@ -5930,9 +6134,15 @@
       <c r="P7" s="7">
         <v>13.3</v>
       </c>
-      <c r="Q7" s="6"/>
-      <c r="R7" s="6"/>
-      <c r="S7" s="6"/>
+      <c r="Q7" s="6">
+        <v>6</v>
+      </c>
+      <c r="R7" s="6">
+        <v>451</v>
+      </c>
+      <c r="S7" s="7">
+        <v>13.3</v>
+      </c>
       <c r="T7" s="6"/>
       <c r="U7" s="6"/>
       <c r="V7" s="6"/>
@@ -5960,7 +6170,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="10">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D8" s="8">
         <v>0</v>
@@ -5969,7 +6179,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G8" s="8">
         <v>0</v>
@@ -5978,7 +6188,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8" s="8">
         <v>0</v>
@@ -5987,7 +6197,7 @@
         <v>0</v>
       </c>
       <c r="L8" s="10">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="M8" s="8">
         <v>0</v>
@@ -5996,14 +6206,20 @@
         <v>0</v>
       </c>
       <c r="O8" s="10">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="P8" s="8">
         <v>0</v>
       </c>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="10"/>
-      <c r="S8" s="10"/>
+      <c r="Q8" s="10">
+        <v>0</v>
+      </c>
+      <c r="R8" s="10">
+        <v>0</v>
+      </c>
+      <c r="S8" s="8">
+        <v>0</v>
+      </c>
       <c r="T8" s="10"/>
       <c r="U8" s="10"/>
       <c r="V8" s="10"/>
@@ -6072,9 +6288,15 @@
       <c r="P9" s="8">
         <v>0</v>
       </c>
-      <c r="Q9" s="6"/>
-      <c r="R9" s="6"/>
-      <c r="S9" s="6"/>
+      <c r="Q9" s="6">
+        <v>0</v>
+      </c>
+      <c r="R9" s="6">
+        <v>0</v>
+      </c>
+      <c r="S9" s="8">
+        <v>0</v>
+      </c>
       <c r="T9" s="6"/>
       <c r="U9" s="6"/>
       <c r="V9" s="6"/>
@@ -6143,9 +6365,15 @@
       <c r="P10" s="8">
         <v>0</v>
       </c>
-      <c r="Q10" s="10"/>
-      <c r="R10" s="10"/>
-      <c r="S10" s="10"/>
+      <c r="Q10" s="10">
+        <v>0</v>
+      </c>
+      <c r="R10" s="10">
+        <v>486</v>
+      </c>
+      <c r="S10" s="8">
+        <v>0</v>
+      </c>
       <c r="T10" s="10"/>
       <c r="U10" s="10"/>
       <c r="V10" s="10"/>
@@ -6214,9 +6442,15 @@
       <c r="P11" s="8">
         <v>0</v>
       </c>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
+      <c r="Q11" s="6">
+        <v>0</v>
+      </c>
+      <c r="R11" s="6">
+        <v>5</v>
+      </c>
+      <c r="S11" s="8">
+        <v>0</v>
+      </c>
       <c r="T11" s="6"/>
       <c r="U11" s="6"/>
       <c r="V11" s="6"/>
@@ -6285,9 +6519,15 @@
       <c r="P12" s="8">
         <v>0</v>
       </c>
-      <c r="Q12" s="10"/>
-      <c r="R12" s="10"/>
-      <c r="S12" s="10"/>
+      <c r="Q12" s="10">
+        <v>3</v>
+      </c>
+      <c r="R12" s="10">
+        <v>0</v>
+      </c>
+      <c r="S12" s="8">
+        <v>0</v>
+      </c>
       <c r="T12" s="10"/>
       <c r="U12" s="10"/>
       <c r="V12" s="10"/>
@@ -6356,9 +6596,15 @@
       <c r="P13" s="8">
         <v>0</v>
       </c>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
-      <c r="S13" s="6"/>
+      <c r="Q13" s="6">
+        <v>0</v>
+      </c>
+      <c r="R13" s="6">
+        <v>0</v>
+      </c>
+      <c r="S13" s="8">
+        <v>0</v>
+      </c>
       <c r="T13" s="6"/>
       <c r="U13" s="6"/>
       <c r="V13" s="6"/>
@@ -6427,9 +6673,15 @@
       <c r="P14" s="8">
         <v>0</v>
       </c>
-      <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
-      <c r="S14" s="10"/>
+      <c r="Q14" s="10">
+        <v>0</v>
+      </c>
+      <c r="R14" s="10">
+        <v>0</v>
+      </c>
+      <c r="S14" s="8">
+        <v>0</v>
+      </c>
       <c r="T14" s="10"/>
       <c r="U14" s="10"/>
       <c r="V14" s="10"/>
@@ -6498,9 +6750,15 @@
       <c r="P15" s="8">
         <v>0</v>
       </c>
-      <c r="Q15" s="6"/>
-      <c r="R15" s="6"/>
-      <c r="S15" s="6"/>
+      <c r="Q15" s="6">
+        <v>0</v>
+      </c>
+      <c r="R15" s="6">
+        <v>0</v>
+      </c>
+      <c r="S15" s="8">
+        <v>0</v>
+      </c>
       <c r="T15" s="6"/>
       <c r="U15" s="6"/>
       <c r="V15" s="6"/>
@@ -6788,9 +7046,15 @@
       <c r="P20" s="7">
         <v>13.51</v>
       </c>
-      <c r="Q20" s="6"/>
-      <c r="R20" s="6"/>
-      <c r="S20" s="6"/>
+      <c r="Q20" s="6">
+        <v>8</v>
+      </c>
+      <c r="R20" s="6">
+        <v>509</v>
+      </c>
+      <c r="S20" s="8">
+        <v>15.72</v>
+      </c>
       <c r="T20" s="6"/>
       <c r="U20" s="6"/>
       <c r="V20" s="6"/>
@@ -6859,9 +7123,15 @@
       <c r="P21" s="7">
         <v>8.26</v>
       </c>
-      <c r="Q21" s="10"/>
-      <c r="R21" s="10"/>
-      <c r="S21" s="10"/>
+      <c r="Q21" s="10">
+        <v>1</v>
+      </c>
+      <c r="R21" s="10">
+        <v>121</v>
+      </c>
+      <c r="S21" s="7">
+        <v>8.26</v>
+      </c>
       <c r="T21" s="10"/>
       <c r="U21" s="10"/>
       <c r="V21" s="10"/>
@@ -6930,9 +7200,15 @@
       <c r="P22" s="7">
         <v>10.14</v>
       </c>
-      <c r="Q22" s="6"/>
-      <c r="R22" s="6"/>
-      <c r="S22" s="6"/>
+      <c r="Q22" s="6">
+        <v>29</v>
+      </c>
+      <c r="R22" s="6">
+        <v>2719</v>
+      </c>
+      <c r="S22" s="7">
+        <v>10.67</v>
+      </c>
       <c r="T22" s="6"/>
       <c r="U22" s="6"/>
       <c r="V22" s="6"/>
@@ -6956,51 +7232,21 @@
       <c r="A23" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="10">
-        <v>0</v>
-      </c>
-      <c r="C23" s="10">
-        <v>10</v>
-      </c>
-      <c r="D23" s="8">
-        <v>0</v>
-      </c>
-      <c r="E23" s="10">
-        <v>0</v>
-      </c>
-      <c r="F23" s="10">
-        <v>13</v>
-      </c>
-      <c r="G23" s="8">
-        <v>0</v>
-      </c>
-      <c r="H23" s="10">
-        <v>0</v>
-      </c>
-      <c r="I23" s="10">
-        <v>14</v>
-      </c>
-      <c r="J23" s="8">
-        <v>0</v>
-      </c>
-      <c r="K23" s="10">
-        <v>0</v>
-      </c>
-      <c r="L23" s="10">
-        <v>27</v>
-      </c>
-      <c r="M23" s="8">
-        <v>0</v>
-      </c>
-      <c r="N23" s="10">
-        <v>0</v>
-      </c>
-      <c r="O23" s="10">
-        <v>36</v>
-      </c>
-      <c r="P23" s="8">
-        <v>0</v>
-      </c>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10"/>
       <c r="Q23" s="10"/>
       <c r="R23" s="10"/>
       <c r="S23" s="10"/>
@@ -7072,9 +7318,15 @@
       <c r="P24" s="8">
         <v>0</v>
       </c>
-      <c r="Q24" s="6"/>
-      <c r="R24" s="6"/>
-      <c r="S24" s="6"/>
+      <c r="Q24" s="6">
+        <v>0</v>
+      </c>
+      <c r="R24" s="6">
+        <v>0</v>
+      </c>
+      <c r="S24" s="8">
+        <v>0</v>
+      </c>
       <c r="T24" s="6"/>
       <c r="U24" s="6"/>
       <c r="V24" s="6"/>
@@ -7143,9 +7395,15 @@
       <c r="P25" s="8">
         <v>3.97</v>
       </c>
-      <c r="Q25" s="10"/>
-      <c r="R25" s="10"/>
-      <c r="S25" s="10"/>
+      <c r="Q25" s="10">
+        <v>12</v>
+      </c>
+      <c r="R25" s="10">
+        <v>3510</v>
+      </c>
+      <c r="S25" s="8">
+        <v>3.42</v>
+      </c>
       <c r="T25" s="10"/>
       <c r="U25" s="10"/>
       <c r="V25" s="10"/>
@@ -7214,9 +7472,15 @@
       <c r="P26" s="8">
         <v>0</v>
       </c>
-      <c r="Q26" s="6"/>
-      <c r="R26" s="6"/>
-      <c r="S26" s="6"/>
+      <c r="Q26" s="6">
+        <v>0</v>
+      </c>
+      <c r="R26" s="6">
+        <v>36</v>
+      </c>
+      <c r="S26" s="8">
+        <v>0</v>
+      </c>
       <c r="T26" s="6"/>
       <c r="U26" s="6"/>
       <c r="V26" s="6"/>
@@ -7285,9 +7549,15 @@
       <c r="P27" s="8">
         <v>27.31</v>
       </c>
-      <c r="Q27" s="10"/>
-      <c r="R27" s="10"/>
-      <c r="S27" s="10"/>
+      <c r="Q27" s="10">
+        <v>47</v>
+      </c>
+      <c r="R27" s="10">
+        <v>1611</v>
+      </c>
+      <c r="S27" s="8">
+        <v>29.17</v>
+      </c>
       <c r="T27" s="10"/>
       <c r="U27" s="10"/>
       <c r="V27" s="10"/>
@@ -7356,9 +7626,15 @@
       <c r="P28" s="8">
         <v>0</v>
       </c>
-      <c r="Q28" s="6"/>
-      <c r="R28" s="6"/>
-      <c r="S28" s="6"/>
+      <c r="Q28" s="6">
+        <v>0</v>
+      </c>
+      <c r="R28" s="6">
+        <v>0</v>
+      </c>
+      <c r="S28" s="8">
+        <v>0</v>
+      </c>
       <c r="T28" s="6"/>
       <c r="U28" s="6"/>
       <c r="V28" s="6"/>
@@ -7427,9 +7703,15 @@
       <c r="P29" s="8">
         <v>0</v>
       </c>
-      <c r="Q29" s="10"/>
-      <c r="R29" s="10"/>
-      <c r="S29" s="10"/>
+      <c r="Q29" s="10">
+        <v>0</v>
+      </c>
+      <c r="R29" s="10">
+        <v>0</v>
+      </c>
+      <c r="S29" s="8">
+        <v>0</v>
+      </c>
       <c r="T29" s="10"/>
       <c r="U29" s="10"/>
       <c r="V29" s="10"/>
@@ -7498,9 +7780,15 @@
       <c r="P30" s="8">
         <v>0</v>
       </c>
-      <c r="Q30" s="6"/>
-      <c r="R30" s="6"/>
-      <c r="S30" s="6"/>
+      <c r="Q30" s="6">
+        <v>0</v>
+      </c>
+      <c r="R30" s="6">
+        <v>0</v>
+      </c>
+      <c r="S30" s="8">
+        <v>0</v>
+      </c>
       <c r="T30" s="6"/>
       <c r="U30" s="6"/>
       <c r="V30" s="6"/>
@@ -7528,50 +7816,56 @@
         <v>24</v>
       </c>
       <c r="C31" s="11">
-        <v>1814</v>
+        <v>1804</v>
       </c>
       <c r="D31" s="7">
-        <v>13.23</v>
+        <v>13.3</v>
       </c>
       <c r="E31" s="11">
         <v>42</v>
       </c>
       <c r="F31" s="11">
-        <v>3746</v>
+        <v>3733</v>
       </c>
       <c r="G31" s="7">
-        <v>11.21</v>
+        <v>11.25</v>
       </c>
       <c r="H31" s="11">
         <v>58</v>
       </c>
       <c r="I31" s="11">
-        <v>5311</v>
+        <v>5297</v>
       </c>
       <c r="J31" s="7">
-        <v>10.92</v>
+        <v>10.95</v>
       </c>
       <c r="K31" s="11">
         <v>75</v>
       </c>
       <c r="L31" s="11">
-        <v>6519</v>
+        <v>6492</v>
       </c>
       <c r="M31" s="7">
-        <v>11.5</v>
+        <v>11.55</v>
       </c>
       <c r="N31" s="11">
         <v>86</v>
       </c>
       <c r="O31" s="11">
-        <v>7535</v>
+        <v>7499</v>
       </c>
       <c r="P31" s="7">
-        <v>11.41</v>
-      </c>
-      <c r="Q31" s="11"/>
-      <c r="R31" s="11"/>
-      <c r="S31" s="11"/>
+        <v>11.47</v>
+      </c>
+      <c r="Q31" s="11">
+        <v>97</v>
+      </c>
+      <c r="R31" s="11">
+        <v>8506</v>
+      </c>
+      <c r="S31" s="7">
+        <v>11.4</v>
+      </c>
       <c r="T31" s="11"/>
       <c r="U31" s="11"/>
       <c r="V31" s="11"/>
@@ -7969,9 +8263,15 @@
       <c r="P5" s="8">
         <v>4.33</v>
       </c>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="6"/>
+      <c r="Q5" s="6">
+        <v>1</v>
+      </c>
+      <c r="R5" s="6">
+        <v>231</v>
+      </c>
+      <c r="S5" s="8">
+        <v>4.33</v>
+      </c>
       <c r="T5" s="6"/>
       <c r="U5" s="6"/>
       <c r="V5" s="6"/>
@@ -8040,9 +8340,15 @@
       <c r="P6" s="8">
         <v>0</v>
       </c>
-      <c r="Q6" s="10"/>
-      <c r="R6" s="10"/>
-      <c r="S6" s="10"/>
+      <c r="Q6" s="10">
+        <v>0</v>
+      </c>
+      <c r="R6" s="10">
+        <v>0</v>
+      </c>
+      <c r="S6" s="8">
+        <v>0</v>
+      </c>
       <c r="T6" s="10"/>
       <c r="U6" s="10"/>
       <c r="V6" s="10"/>
@@ -8111,9 +8417,15 @@
       <c r="P7" s="8">
         <v>0</v>
       </c>
-      <c r="Q7" s="6"/>
-      <c r="R7" s="6"/>
-      <c r="S7" s="6"/>
+      <c r="Q7" s="6">
+        <v>0</v>
+      </c>
+      <c r="R7" s="6">
+        <v>963</v>
+      </c>
+      <c r="S7" s="8">
+        <v>0</v>
+      </c>
       <c r="T7" s="6"/>
       <c r="U7" s="6"/>
       <c r="V7" s="6"/>
@@ -8141,7 +8453,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="10">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="D8" s="8">
         <v>0</v>
@@ -8150,7 +8462,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="10">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="G8" s="8">
         <v>0</v>
@@ -8159,7 +8471,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="10">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="J8" s="8">
         <v>0</v>
@@ -8168,7 +8480,7 @@
         <v>0</v>
       </c>
       <c r="L8" s="10">
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="M8" s="8">
         <v>0</v>
@@ -8177,14 +8489,20 @@
         <v>0</v>
       </c>
       <c r="O8" s="10">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="P8" s="8">
         <v>0</v>
       </c>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="10"/>
-      <c r="S8" s="10"/>
+      <c r="Q8" s="10">
+        <v>0</v>
+      </c>
+      <c r="R8" s="10">
+        <v>0</v>
+      </c>
+      <c r="S8" s="8">
+        <v>0</v>
+      </c>
       <c r="T8" s="10"/>
       <c r="U8" s="10"/>
       <c r="V8" s="10"/>
@@ -8253,9 +8571,15 @@
       <c r="P9" s="8">
         <v>0</v>
       </c>
-      <c r="Q9" s="6"/>
-      <c r="R9" s="6"/>
-      <c r="S9" s="6"/>
+      <c r="Q9" s="6">
+        <v>0</v>
+      </c>
+      <c r="R9" s="6">
+        <v>0</v>
+      </c>
+      <c r="S9" s="8">
+        <v>0</v>
+      </c>
       <c r="T9" s="6"/>
       <c r="U9" s="6"/>
       <c r="V9" s="6"/>
@@ -8324,9 +8648,15 @@
       <c r="P10" s="7">
         <v>2.04</v>
       </c>
-      <c r="Q10" s="10"/>
-      <c r="R10" s="10"/>
-      <c r="S10" s="10"/>
+      <c r="Q10" s="10">
+        <v>3</v>
+      </c>
+      <c r="R10" s="10">
+        <v>1468</v>
+      </c>
+      <c r="S10" s="7">
+        <v>2.04</v>
+      </c>
       <c r="T10" s="10"/>
       <c r="U10" s="10"/>
       <c r="V10" s="10"/>
@@ -8395,9 +8725,15 @@
       <c r="P11" s="8">
         <v>0</v>
       </c>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
+      <c r="Q11" s="6">
+        <v>0</v>
+      </c>
+      <c r="R11" s="6">
+        <v>68</v>
+      </c>
+      <c r="S11" s="8">
+        <v>0</v>
+      </c>
       <c r="T11" s="6"/>
       <c r="U11" s="6"/>
       <c r="V11" s="6"/>
@@ -8466,9 +8802,15 @@
       <c r="P12" s="8">
         <v>0</v>
       </c>
-      <c r="Q12" s="10"/>
-      <c r="R12" s="10"/>
-      <c r="S12" s="10"/>
+      <c r="Q12" s="10">
+        <v>0</v>
+      </c>
+      <c r="R12" s="10">
+        <v>0</v>
+      </c>
+      <c r="S12" s="8">
+        <v>0</v>
+      </c>
       <c r="T12" s="10"/>
       <c r="U12" s="10"/>
       <c r="V12" s="10"/>
@@ -8537,9 +8879,15 @@
       <c r="P13" s="8">
         <v>0</v>
       </c>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
-      <c r="S13" s="6"/>
+      <c r="Q13" s="6">
+        <v>0</v>
+      </c>
+      <c r="R13" s="6">
+        <v>0</v>
+      </c>
+      <c r="S13" s="8">
+        <v>0</v>
+      </c>
       <c r="T13" s="6"/>
       <c r="U13" s="6"/>
       <c r="V13" s="6"/>
@@ -8608,9 +8956,15 @@
       <c r="P14" s="8">
         <v>0</v>
       </c>
-      <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
-      <c r="S14" s="10"/>
+      <c r="Q14" s="10">
+        <v>0</v>
+      </c>
+      <c r="R14" s="10">
+        <v>0</v>
+      </c>
+      <c r="S14" s="8">
+        <v>0</v>
+      </c>
       <c r="T14" s="10"/>
       <c r="U14" s="10"/>
       <c r="V14" s="10"/>
@@ -8679,9 +9033,15 @@
       <c r="P15" s="8">
         <v>0</v>
       </c>
-      <c r="Q15" s="6"/>
-      <c r="R15" s="6"/>
-      <c r="S15" s="6"/>
+      <c r="Q15" s="6">
+        <v>0</v>
+      </c>
+      <c r="R15" s="6">
+        <v>0</v>
+      </c>
+      <c r="S15" s="8">
+        <v>0</v>
+      </c>
       <c r="T15" s="6"/>
       <c r="U15" s="6"/>
       <c r="V15" s="6"/>
@@ -8969,9 +9329,15 @@
       <c r="P20" s="7">
         <v>2.23</v>
       </c>
-      <c r="Q20" s="6"/>
-      <c r="R20" s="6"/>
-      <c r="S20" s="6"/>
+      <c r="Q20" s="6">
+        <v>4</v>
+      </c>
+      <c r="R20" s="6">
+        <v>1574</v>
+      </c>
+      <c r="S20" s="7">
+        <v>2.54</v>
+      </c>
       <c r="T20" s="6"/>
       <c r="U20" s="6"/>
       <c r="V20" s="6"/>
@@ -9040,9 +9406,15 @@
       <c r="P21" s="8">
         <v>7.32</v>
       </c>
-      <c r="Q21" s="10"/>
-      <c r="R21" s="10"/>
-      <c r="S21" s="10"/>
+      <c r="Q21" s="10">
+        <v>3</v>
+      </c>
+      <c r="R21" s="10">
+        <v>410</v>
+      </c>
+      <c r="S21" s="8">
+        <v>7.32</v>
+      </c>
       <c r="T21" s="10"/>
       <c r="U21" s="10"/>
       <c r="V21" s="10"/>
@@ -9111,9 +9483,15 @@
       <c r="P22" s="8">
         <v>0</v>
       </c>
-      <c r="Q22" s="6"/>
-      <c r="R22" s="6"/>
-      <c r="S22" s="6"/>
+      <c r="Q22" s="6">
+        <v>0</v>
+      </c>
+      <c r="R22" s="6">
+        <v>4981</v>
+      </c>
+      <c r="S22" s="8">
+        <v>0</v>
+      </c>
       <c r="T22" s="6"/>
       <c r="U22" s="6"/>
       <c r="V22" s="6"/>
@@ -9137,51 +9515,21 @@
       <c r="A23" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="10">
-        <v>0</v>
-      </c>
-      <c r="C23" s="10">
-        <v>41</v>
-      </c>
-      <c r="D23" s="8">
-        <v>0</v>
-      </c>
-      <c r="E23" s="10">
-        <v>0</v>
-      </c>
-      <c r="F23" s="10">
-        <v>82</v>
-      </c>
-      <c r="G23" s="8">
-        <v>0</v>
-      </c>
-      <c r="H23" s="10">
-        <v>0</v>
-      </c>
-      <c r="I23" s="10">
-        <v>147</v>
-      </c>
-      <c r="J23" s="8">
-        <v>0</v>
-      </c>
-      <c r="K23" s="10">
-        <v>0</v>
-      </c>
-      <c r="L23" s="10">
-        <v>226</v>
-      </c>
-      <c r="M23" s="8">
-        <v>0</v>
-      </c>
-      <c r="N23" s="10">
-        <v>0</v>
-      </c>
-      <c r="O23" s="10">
-        <v>269</v>
-      </c>
-      <c r="P23" s="8">
-        <v>0</v>
-      </c>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10"/>
       <c r="Q23" s="10"/>
       <c r="R23" s="10"/>
       <c r="S23" s="10"/>
@@ -9253,9 +9601,15 @@
       <c r="P24" s="8">
         <v>0</v>
       </c>
-      <c r="Q24" s="6"/>
-      <c r="R24" s="6"/>
-      <c r="S24" s="6"/>
+      <c r="Q24" s="6">
+        <v>0</v>
+      </c>
+      <c r="R24" s="6">
+        <v>0</v>
+      </c>
+      <c r="S24" s="8">
+        <v>0</v>
+      </c>
       <c r="T24" s="6"/>
       <c r="U24" s="6"/>
       <c r="V24" s="6"/>
@@ -9324,9 +9678,15 @@
       <c r="P25" s="8">
         <v>0.59</v>
       </c>
-      <c r="Q25" s="10"/>
-      <c r="R25" s="10"/>
-      <c r="S25" s="10"/>
+      <c r="Q25" s="10">
+        <v>9</v>
+      </c>
+      <c r="R25" s="10">
+        <v>11634</v>
+      </c>
+      <c r="S25" s="8">
+        <v>0.77</v>
+      </c>
       <c r="T25" s="10"/>
       <c r="U25" s="10"/>
       <c r="V25" s="10"/>
@@ -9395,9 +9755,15 @@
       <c r="P26" s="8">
         <v>0</v>
       </c>
-      <c r="Q26" s="6"/>
-      <c r="R26" s="6"/>
-      <c r="S26" s="6"/>
+      <c r="Q26" s="6">
+        <v>0</v>
+      </c>
+      <c r="R26" s="6">
+        <v>265</v>
+      </c>
+      <c r="S26" s="8">
+        <v>0</v>
+      </c>
       <c r="T26" s="6"/>
       <c r="U26" s="6"/>
       <c r="V26" s="6"/>
@@ -9466,9 +9832,15 @@
       <c r="P27" s="7">
         <v>1.82</v>
       </c>
-      <c r="Q27" s="10"/>
-      <c r="R27" s="10"/>
-      <c r="S27" s="10"/>
+      <c r="Q27" s="10">
+        <v>6</v>
+      </c>
+      <c r="R27" s="10">
+        <v>3305</v>
+      </c>
+      <c r="S27" s="7">
+        <v>1.82</v>
+      </c>
       <c r="T27" s="10"/>
       <c r="U27" s="10"/>
       <c r="V27" s="10"/>
@@ -9537,9 +9909,15 @@
       <c r="P28" s="8">
         <v>0</v>
       </c>
-      <c r="Q28" s="6"/>
-      <c r="R28" s="6"/>
-      <c r="S28" s="6"/>
+      <c r="Q28" s="6">
+        <v>0</v>
+      </c>
+      <c r="R28" s="6">
+        <v>0</v>
+      </c>
+      <c r="S28" s="8">
+        <v>0</v>
+      </c>
       <c r="T28" s="6"/>
       <c r="U28" s="6"/>
       <c r="V28" s="6"/>
@@ -9608,9 +9986,15 @@
       <c r="P29" s="8">
         <v>0</v>
       </c>
-      <c r="Q29" s="10"/>
-      <c r="R29" s="10"/>
-      <c r="S29" s="10"/>
+      <c r="Q29" s="10">
+        <v>0</v>
+      </c>
+      <c r="R29" s="10">
+        <v>0</v>
+      </c>
+      <c r="S29" s="8">
+        <v>0</v>
+      </c>
       <c r="T29" s="10"/>
       <c r="U29" s="10"/>
       <c r="V29" s="10"/>
@@ -9679,9 +10063,15 @@
       <c r="P30" s="8">
         <v>0</v>
       </c>
-      <c r="Q30" s="6"/>
-      <c r="R30" s="6"/>
-      <c r="S30" s="6"/>
+      <c r="Q30" s="6">
+        <v>0</v>
+      </c>
+      <c r="R30" s="6">
+        <v>0</v>
+      </c>
+      <c r="S30" s="8">
+        <v>0</v>
+      </c>
       <c r="T30" s="6"/>
       <c r="U30" s="6"/>
       <c r="V30" s="6"/>
@@ -9709,50 +10099,56 @@
         <v>6</v>
       </c>
       <c r="C31" s="11">
-        <v>3871</v>
+        <v>3830</v>
       </c>
       <c r="D31" s="7">
-        <v>1.55</v>
+        <v>1.57</v>
       </c>
       <c r="E31" s="11">
         <v>8</v>
       </c>
       <c r="F31" s="11">
-        <v>8799</v>
+        <v>8717</v>
       </c>
       <c r="G31" s="8">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="H31" s="11">
         <v>11</v>
       </c>
       <c r="I31" s="11">
-        <v>12896</v>
+        <v>12749</v>
       </c>
       <c r="J31" s="8">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="K31" s="11">
         <v>14</v>
       </c>
       <c r="L31" s="11">
-        <v>16935</v>
+        <v>16709</v>
       </c>
       <c r="M31" s="8">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="N31" s="11">
         <v>18</v>
       </c>
       <c r="O31" s="11">
-        <v>19708</v>
+        <v>19439</v>
       </c>
       <c r="P31" s="8">
-        <v>0.91</v>
-      </c>
-      <c r="Q31" s="11"/>
-      <c r="R31" s="11"/>
-      <c r="S31" s="11"/>
+        <v>0.93</v>
+      </c>
+      <c r="Q31" s="11">
+        <v>22</v>
+      </c>
+      <c r="R31" s="11">
+        <v>22169</v>
+      </c>
+      <c r="S31" s="8">
+        <v>0.99</v>
+      </c>
       <c r="T31" s="11"/>
       <c r="U31" s="11"/>
       <c r="V31" s="11"/>
@@ -10150,9 +10546,15 @@
       <c r="P5" s="7">
         <v>12.69</v>
       </c>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="6"/>
+      <c r="Q5" s="6">
+        <v>5</v>
+      </c>
+      <c r="R5" s="6">
+        <v>394</v>
+      </c>
+      <c r="S5" s="7">
+        <v>12.69</v>
+      </c>
       <c r="T5" s="6"/>
       <c r="U5" s="6"/>
       <c r="V5" s="6"/>
@@ -10221,9 +10623,15 @@
       <c r="P6" s="8">
         <v>0</v>
       </c>
-      <c r="Q6" s="10"/>
-      <c r="R6" s="10"/>
-      <c r="S6" s="10"/>
+      <c r="Q6" s="10">
+        <v>3</v>
+      </c>
+      <c r="R6" s="10">
+        <v>0</v>
+      </c>
+      <c r="S6" s="8">
+        <v>0</v>
+      </c>
       <c r="T6" s="10"/>
       <c r="U6" s="10"/>
       <c r="V6" s="10"/>
@@ -10292,9 +10700,15 @@
       <c r="P7" s="7">
         <v>5.35</v>
       </c>
-      <c r="Q7" s="6"/>
-      <c r="R7" s="6"/>
-      <c r="S7" s="6"/>
+      <c r="Q7" s="6">
+        <v>5</v>
+      </c>
+      <c r="R7" s="6">
+        <v>935</v>
+      </c>
+      <c r="S7" s="7">
+        <v>5.35</v>
+      </c>
       <c r="T7" s="6"/>
       <c r="U7" s="6"/>
       <c r="V7" s="6"/>
@@ -10319,19 +10733,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8" s="10">
-        <v>78</v>
-      </c>
-      <c r="D8" s="7">
-        <v>12.8205</v>
+        <v>0</v>
+      </c>
+      <c r="D8" s="8">
+        <v>0</v>
       </c>
       <c r="E8" s="10">
         <v>0</v>
       </c>
       <c r="F8" s="10">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="G8" s="8">
         <v>0</v>
@@ -10340,7 +10754,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="10">
-        <v>111</v>
+        <v>0</v>
       </c>
       <c r="J8" s="8">
         <v>0</v>
@@ -10349,7 +10763,7 @@
         <v>0</v>
       </c>
       <c r="L8" s="10">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="M8" s="8">
         <v>0</v>
@@ -10358,14 +10772,20 @@
         <v>0</v>
       </c>
       <c r="O8" s="10">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="P8" s="8">
         <v>0</v>
       </c>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="10"/>
-      <c r="S8" s="10"/>
+      <c r="Q8" s="10">
+        <v>0</v>
+      </c>
+      <c r="R8" s="10">
+        <v>0</v>
+      </c>
+      <c r="S8" s="8">
+        <v>0</v>
+      </c>
       <c r="T8" s="10"/>
       <c r="U8" s="10"/>
       <c r="V8" s="10"/>
@@ -10434,9 +10854,15 @@
       <c r="P9" s="8">
         <v>0</v>
       </c>
-      <c r="Q9" s="6"/>
-      <c r="R9" s="6"/>
-      <c r="S9" s="6"/>
+      <c r="Q9" s="6">
+        <v>0</v>
+      </c>
+      <c r="R9" s="6">
+        <v>0</v>
+      </c>
+      <c r="S9" s="8">
+        <v>0</v>
+      </c>
       <c r="T9" s="6"/>
       <c r="U9" s="6"/>
       <c r="V9" s="6"/>
@@ -10505,9 +10931,15 @@
       <c r="P10" s="9">
         <v>1.47</v>
       </c>
-      <c r="Q10" s="10"/>
-      <c r="R10" s="10"/>
-      <c r="S10" s="10"/>
+      <c r="Q10" s="10">
+        <v>2</v>
+      </c>
+      <c r="R10" s="10">
+        <v>1360</v>
+      </c>
+      <c r="S10" s="9">
+        <v>1.47</v>
+      </c>
       <c r="T10" s="10"/>
       <c r="U10" s="10"/>
       <c r="V10" s="10"/>
@@ -10576,9 +11008,15 @@
       <c r="P11" s="8">
         <v>0</v>
       </c>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
+      <c r="Q11" s="6">
+        <v>0</v>
+      </c>
+      <c r="R11" s="6">
+        <v>102</v>
+      </c>
+      <c r="S11" s="8">
+        <v>0</v>
+      </c>
       <c r="T11" s="6"/>
       <c r="U11" s="6"/>
       <c r="V11" s="6"/>
@@ -10647,9 +11085,15 @@
       <c r="P12" s="8">
         <v>0</v>
       </c>
-      <c r="Q12" s="10"/>
-      <c r="R12" s="10"/>
-      <c r="S12" s="10"/>
+      <c r="Q12" s="10">
+        <v>4</v>
+      </c>
+      <c r="R12" s="10">
+        <v>0</v>
+      </c>
+      <c r="S12" s="8">
+        <v>0</v>
+      </c>
       <c r="T12" s="10"/>
       <c r="U12" s="10"/>
       <c r="V12" s="10"/>
@@ -10718,9 +11162,15 @@
       <c r="P13" s="8">
         <v>0</v>
       </c>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
-      <c r="S13" s="6"/>
+      <c r="Q13" s="6">
+        <v>0</v>
+      </c>
+      <c r="R13" s="6">
+        <v>0</v>
+      </c>
+      <c r="S13" s="8">
+        <v>0</v>
+      </c>
       <c r="T13" s="6"/>
       <c r="U13" s="6"/>
       <c r="V13" s="6"/>
@@ -10789,9 +11239,15 @@
       <c r="P14" s="8">
         <v>0</v>
       </c>
-      <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
-      <c r="S14" s="10"/>
+      <c r="Q14" s="10">
+        <v>0</v>
+      </c>
+      <c r="R14" s="10">
+        <v>0</v>
+      </c>
+      <c r="S14" s="8">
+        <v>0</v>
+      </c>
       <c r="T14" s="10"/>
       <c r="U14" s="10"/>
       <c r="V14" s="10"/>
@@ -10860,9 +11316,15 @@
       <c r="P15" s="8">
         <v>0</v>
       </c>
-      <c r="Q15" s="6"/>
-      <c r="R15" s="6"/>
-      <c r="S15" s="6"/>
+      <c r="Q15" s="6">
+        <v>0</v>
+      </c>
+      <c r="R15" s="6">
+        <v>0</v>
+      </c>
+      <c r="S15" s="8">
+        <v>0</v>
+      </c>
       <c r="T15" s="6"/>
       <c r="U15" s="6"/>
       <c r="V15" s="6"/>
@@ -11150,9 +11612,15 @@
       <c r="P20" s="7">
         <v>10.29</v>
       </c>
-      <c r="Q20" s="6"/>
-      <c r="R20" s="6"/>
-      <c r="S20" s="6"/>
+      <c r="Q20" s="6">
+        <v>32</v>
+      </c>
+      <c r="R20" s="6">
+        <v>3018</v>
+      </c>
+      <c r="S20" s="7">
+        <v>10.6</v>
+      </c>
       <c r="T20" s="6"/>
       <c r="U20" s="6"/>
       <c r="V20" s="6"/>
@@ -11221,9 +11689,15 @@
       <c r="P21" s="7">
         <v>10.96</v>
       </c>
-      <c r="Q21" s="10"/>
-      <c r="R21" s="10"/>
-      <c r="S21" s="10"/>
+      <c r="Q21" s="10">
+        <v>13</v>
+      </c>
+      <c r="R21" s="10">
+        <v>912</v>
+      </c>
+      <c r="S21" s="8">
+        <v>14.25</v>
+      </c>
       <c r="T21" s="10"/>
       <c r="U21" s="10"/>
       <c r="V21" s="10"/>
@@ -11292,9 +11766,15 @@
       <c r="P22" s="9">
         <v>1.78</v>
       </c>
-      <c r="Q22" s="6"/>
-      <c r="R22" s="6"/>
-      <c r="S22" s="6"/>
+      <c r="Q22" s="6">
+        <v>20</v>
+      </c>
+      <c r="R22" s="6">
+        <v>9358</v>
+      </c>
+      <c r="S22" s="9">
+        <v>2.14</v>
+      </c>
       <c r="T22" s="6"/>
       <c r="U22" s="6"/>
       <c r="V22" s="6"/>
@@ -11318,51 +11798,21 @@
       <c r="A23" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="10">
-        <v>1</v>
-      </c>
-      <c r="C23" s="10">
-        <v>78</v>
-      </c>
-      <c r="D23" s="7">
-        <v>12.82</v>
-      </c>
-      <c r="E23" s="10">
-        <v>1</v>
-      </c>
-      <c r="F23" s="10">
-        <v>152</v>
-      </c>
-      <c r="G23" s="7">
-        <v>6.58</v>
-      </c>
-      <c r="H23" s="10">
-        <v>1</v>
-      </c>
-      <c r="I23" s="10">
-        <v>263</v>
-      </c>
-      <c r="J23" s="9">
-        <v>3.8</v>
-      </c>
-      <c r="K23" s="10">
-        <v>1</v>
-      </c>
-      <c r="L23" s="10">
-        <v>343</v>
-      </c>
-      <c r="M23" s="9">
-        <v>2.92</v>
-      </c>
-      <c r="N23" s="10">
-        <v>1</v>
-      </c>
-      <c r="O23" s="10">
-        <v>433</v>
-      </c>
-      <c r="P23" s="9">
-        <v>2.31</v>
-      </c>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10"/>
       <c r="Q23" s="10"/>
       <c r="R23" s="10"/>
       <c r="S23" s="10"/>
@@ -11434,9 +11884,15 @@
       <c r="P24" s="8">
         <v>0</v>
       </c>
-      <c r="Q24" s="6"/>
-      <c r="R24" s="6"/>
-      <c r="S24" s="6"/>
+      <c r="Q24" s="6">
+        <v>0</v>
+      </c>
+      <c r="R24" s="6">
+        <v>0</v>
+      </c>
+      <c r="S24" s="8">
+        <v>0</v>
+      </c>
       <c r="T24" s="6"/>
       <c r="U24" s="6"/>
       <c r="V24" s="6"/>
@@ -11505,9 +11961,15 @@
       <c r="P25" s="8">
         <v>0.32</v>
       </c>
-      <c r="Q25" s="10"/>
-      <c r="R25" s="10"/>
-      <c r="S25" s="10"/>
+      <c r="Q25" s="10">
+        <v>5</v>
+      </c>
+      <c r="R25" s="10">
+        <v>10821</v>
+      </c>
+      <c r="S25" s="8">
+        <v>0.46</v>
+      </c>
       <c r="T25" s="10"/>
       <c r="U25" s="10"/>
       <c r="V25" s="10"/>
@@ -11576,9 +12038,15 @@
       <c r="P26" s="7">
         <v>7.08</v>
       </c>
-      <c r="Q26" s="6"/>
-      <c r="R26" s="6"/>
-      <c r="S26" s="6"/>
+      <c r="Q26" s="6">
+        <v>4</v>
+      </c>
+      <c r="R26" s="6">
+        <v>667</v>
+      </c>
+      <c r="S26" s="7">
+        <v>6</v>
+      </c>
       <c r="T26" s="6"/>
       <c r="U26" s="6"/>
       <c r="V26" s="6"/>
@@ -11647,9 +12115,15 @@
       <c r="P27" s="7">
         <v>7.11</v>
       </c>
-      <c r="Q27" s="10"/>
-      <c r="R27" s="10"/>
-      <c r="S27" s="10"/>
+      <c r="Q27" s="10">
+        <v>38</v>
+      </c>
+      <c r="R27" s="10">
+        <v>4781</v>
+      </c>
+      <c r="S27" s="7">
+        <v>7.95</v>
+      </c>
       <c r="T27" s="10"/>
       <c r="U27" s="10"/>
       <c r="V27" s="10"/>
@@ -11718,9 +12192,15 @@
       <c r="P28" s="8">
         <v>0</v>
       </c>
-      <c r="Q28" s="6"/>
-      <c r="R28" s="6"/>
-      <c r="S28" s="6"/>
+      <c r="Q28" s="6">
+        <v>0</v>
+      </c>
+      <c r="R28" s="6">
+        <v>0</v>
+      </c>
+      <c r="S28" s="8">
+        <v>0</v>
+      </c>
       <c r="T28" s="6"/>
       <c r="U28" s="6"/>
       <c r="V28" s="6"/>
@@ -11789,9 +12269,15 @@
       <c r="P29" s="8">
         <v>0</v>
       </c>
-      <c r="Q29" s="10"/>
-      <c r="R29" s="10"/>
-      <c r="S29" s="10"/>
+      <c r="Q29" s="10">
+        <v>0</v>
+      </c>
+      <c r="R29" s="10">
+        <v>0</v>
+      </c>
+      <c r="S29" s="8">
+        <v>0</v>
+      </c>
       <c r="T29" s="10"/>
       <c r="U29" s="10"/>
       <c r="V29" s="10"/>
@@ -11860,9 +12346,15 @@
       <c r="P30" s="8">
         <v>0</v>
       </c>
-      <c r="Q30" s="6"/>
-      <c r="R30" s="6"/>
-      <c r="S30" s="6"/>
+      <c r="Q30" s="6">
+        <v>0</v>
+      </c>
+      <c r="R30" s="6">
+        <v>0</v>
+      </c>
+      <c r="S30" s="8">
+        <v>0</v>
+      </c>
       <c r="T30" s="6"/>
       <c r="U30" s="6"/>
       <c r="V30" s="6"/>
@@ -11887,53 +12379,59 @@
         <v>15</v>
       </c>
       <c r="B31" s="11">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C31" s="11">
-        <v>6087</v>
+        <v>6009</v>
       </c>
       <c r="D31" s="9">
-        <v>3.94</v>
+        <v>3.83</v>
       </c>
       <c r="E31" s="11">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F31" s="11">
-        <v>13575</v>
+        <v>13423</v>
       </c>
       <c r="G31" s="9">
+        <v>3.5</v>
+      </c>
+      <c r="H31" s="11">
+        <v>64</v>
+      </c>
+      <c r="I31" s="11">
+        <v>18060</v>
+      </c>
+      <c r="J31" s="9">
         <v>3.54</v>
       </c>
-      <c r="H31" s="11">
-        <v>65</v>
-      </c>
-      <c r="I31" s="11">
-        <v>18323</v>
-      </c>
-      <c r="J31" s="9">
-        <v>3.55</v>
-      </c>
       <c r="K31" s="11">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L31" s="11">
-        <v>24318</v>
+        <v>23975</v>
       </c>
       <c r="M31" s="9">
-        <v>3.08</v>
+        <v>3.09</v>
       </c>
       <c r="N31" s="11">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="O31" s="11">
-        <v>27199</v>
+        <v>26766</v>
       </c>
       <c r="P31" s="9">
-        <v>3.46</v>
-      </c>
-      <c r="Q31" s="11"/>
-      <c r="R31" s="11"/>
-      <c r="S31" s="11"/>
+        <v>3.47</v>
+      </c>
+      <c r="Q31" s="11">
+        <v>112</v>
+      </c>
+      <c r="R31" s="11">
+        <v>29557</v>
+      </c>
+      <c r="S31" s="9">
+        <v>3.79</v>
+      </c>
       <c r="T31" s="11"/>
       <c r="U31" s="11"/>
       <c r="V31" s="11"/>
@@ -12331,9 +12829,15 @@
       <c r="P5" s="8">
         <v>0</v>
       </c>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="6"/>
+      <c r="Q5" s="6">
+        <v>0</v>
+      </c>
+      <c r="R5" s="6">
+        <v>0</v>
+      </c>
+      <c r="S5" s="8">
+        <v>0</v>
+      </c>
       <c r="T5" s="6"/>
       <c r="U5" s="6"/>
       <c r="V5" s="6"/>
@@ -12402,9 +12906,15 @@
       <c r="P6" s="8">
         <v>0</v>
       </c>
-      <c r="Q6" s="10"/>
-      <c r="R6" s="10"/>
-      <c r="S6" s="10"/>
+      <c r="Q6" s="10">
+        <v>0</v>
+      </c>
+      <c r="R6" s="10">
+        <v>0</v>
+      </c>
+      <c r="S6" s="8">
+        <v>0</v>
+      </c>
       <c r="T6" s="10"/>
       <c r="U6" s="10"/>
       <c r="V6" s="10"/>
@@ -12473,9 +12983,15 @@
       <c r="P7" s="7">
         <v>14.49</v>
       </c>
-      <c r="Q7" s="6"/>
-      <c r="R7" s="6"/>
-      <c r="S7" s="6"/>
+      <c r="Q7" s="6">
+        <v>2</v>
+      </c>
+      <c r="R7" s="6">
+        <v>138</v>
+      </c>
+      <c r="S7" s="7">
+        <v>14.49</v>
+      </c>
       <c r="T7" s="6"/>
       <c r="U7" s="6"/>
       <c r="V7" s="6"/>
@@ -12544,9 +13060,15 @@
       <c r="P8" s="8">
         <v>0</v>
       </c>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="10"/>
-      <c r="S8" s="10"/>
+      <c r="Q8" s="10">
+        <v>0</v>
+      </c>
+      <c r="R8" s="10">
+        <v>0</v>
+      </c>
+      <c r="S8" s="8">
+        <v>0</v>
+      </c>
       <c r="T8" s="10"/>
       <c r="U8" s="10"/>
       <c r="V8" s="10"/>
@@ -12615,9 +13137,15 @@
       <c r="P9" s="8">
         <v>0</v>
       </c>
-      <c r="Q9" s="6"/>
-      <c r="R9" s="6"/>
-      <c r="S9" s="6"/>
+      <c r="Q9" s="6">
+        <v>0</v>
+      </c>
+      <c r="R9" s="6">
+        <v>0</v>
+      </c>
+      <c r="S9" s="8">
+        <v>0</v>
+      </c>
       <c r="T9" s="6"/>
       <c r="U9" s="6"/>
       <c r="V9" s="6"/>
@@ -12686,9 +13214,15 @@
       <c r="P10" s="8">
         <v>0</v>
       </c>
-      <c r="Q10" s="10"/>
-      <c r="R10" s="10"/>
-      <c r="S10" s="10"/>
+      <c r="Q10" s="10">
+        <v>0</v>
+      </c>
+      <c r="R10" s="10">
+        <v>10</v>
+      </c>
+      <c r="S10" s="8">
+        <v>0</v>
+      </c>
       <c r="T10" s="10"/>
       <c r="U10" s="10"/>
       <c r="V10" s="10"/>
@@ -12757,9 +13291,15 @@
       <c r="P11" s="8">
         <v>0</v>
       </c>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
+      <c r="Q11" s="6">
+        <v>0</v>
+      </c>
+      <c r="R11" s="6">
+        <v>0</v>
+      </c>
+      <c r="S11" s="8">
+        <v>0</v>
+      </c>
       <c r="T11" s="6"/>
       <c r="U11" s="6"/>
       <c r="V11" s="6"/>
@@ -12828,9 +13368,15 @@
       <c r="P12" s="8">
         <v>0</v>
       </c>
-      <c r="Q12" s="10"/>
-      <c r="R12" s="10"/>
-      <c r="S12" s="10"/>
+      <c r="Q12" s="10">
+        <v>0</v>
+      </c>
+      <c r="R12" s="10">
+        <v>0</v>
+      </c>
+      <c r="S12" s="8">
+        <v>0</v>
+      </c>
       <c r="T12" s="10"/>
       <c r="U12" s="10"/>
       <c r="V12" s="10"/>
@@ -12899,9 +13445,15 @@
       <c r="P13" s="8">
         <v>0</v>
       </c>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
-      <c r="S13" s="6"/>
+      <c r="Q13" s="6">
+        <v>0</v>
+      </c>
+      <c r="R13" s="6">
+        <v>0</v>
+      </c>
+      <c r="S13" s="8">
+        <v>0</v>
+      </c>
       <c r="T13" s="6"/>
       <c r="U13" s="6"/>
       <c r="V13" s="6"/>
@@ -12970,9 +13522,15 @@
       <c r="P14" s="8">
         <v>0</v>
       </c>
-      <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
-      <c r="S14" s="10"/>
+      <c r="Q14" s="10">
+        <v>0</v>
+      </c>
+      <c r="R14" s="10">
+        <v>0</v>
+      </c>
+      <c r="S14" s="8">
+        <v>0</v>
+      </c>
       <c r="T14" s="10"/>
       <c r="U14" s="10"/>
       <c r="V14" s="10"/>
@@ -13041,9 +13599,15 @@
       <c r="P15" s="8">
         <v>0</v>
       </c>
-      <c r="Q15" s="6"/>
-      <c r="R15" s="6"/>
-      <c r="S15" s="6"/>
+      <c r="Q15" s="6">
+        <v>0</v>
+      </c>
+      <c r="R15" s="6">
+        <v>0</v>
+      </c>
+      <c r="S15" s="8">
+        <v>0</v>
+      </c>
       <c r="T15" s="6"/>
       <c r="U15" s="6"/>
       <c r="V15" s="6"/>
@@ -13331,9 +13895,15 @@
       <c r="P20" s="7">
         <v>14.08</v>
       </c>
-      <c r="Q20" s="6"/>
-      <c r="R20" s="6"/>
-      <c r="S20" s="6"/>
+      <c r="Q20" s="6">
+        <v>2</v>
+      </c>
+      <c r="R20" s="6">
+        <v>142</v>
+      </c>
+      <c r="S20" s="7">
+        <v>14.08</v>
+      </c>
       <c r="T20" s="6"/>
       <c r="U20" s="6"/>
       <c r="V20" s="6"/>
@@ -13402,9 +13972,15 @@
       <c r="P21" s="8">
         <v>0</v>
       </c>
-      <c r="Q21" s="10"/>
-      <c r="R21" s="10"/>
-      <c r="S21" s="10"/>
+      <c r="Q21" s="10">
+        <v>0</v>
+      </c>
+      <c r="R21" s="10">
+        <v>0</v>
+      </c>
+      <c r="S21" s="8">
+        <v>0</v>
+      </c>
       <c r="T21" s="10"/>
       <c r="U21" s="10"/>
       <c r="V21" s="10"/>
@@ -13473,9 +14049,15 @@
       <c r="P22" s="7">
         <v>16.82</v>
       </c>
-      <c r="Q22" s="6"/>
-      <c r="R22" s="6"/>
-      <c r="S22" s="6"/>
+      <c r="Q22" s="6">
+        <v>15</v>
+      </c>
+      <c r="R22" s="6">
+        <v>911</v>
+      </c>
+      <c r="S22" s="7">
+        <v>16.47</v>
+      </c>
       <c r="T22" s="6"/>
       <c r="U22" s="6"/>
       <c r="V22" s="6"/>
@@ -13499,51 +14081,21 @@
       <c r="A23" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="10">
-        <v>0</v>
-      </c>
-      <c r="C23" s="10">
-        <v>0</v>
-      </c>
-      <c r="D23" s="8">
-        <v>0</v>
-      </c>
-      <c r="E23" s="10">
-        <v>0</v>
-      </c>
-      <c r="F23" s="10">
-        <v>0</v>
-      </c>
-      <c r="G23" s="8">
-        <v>0</v>
-      </c>
-      <c r="H23" s="10">
-        <v>0</v>
-      </c>
-      <c r="I23" s="10">
-        <v>0</v>
-      </c>
-      <c r="J23" s="8">
-        <v>0</v>
-      </c>
-      <c r="K23" s="10">
-        <v>0</v>
-      </c>
-      <c r="L23" s="10">
-        <v>0</v>
-      </c>
-      <c r="M23" s="8">
-        <v>0</v>
-      </c>
-      <c r="N23" s="10">
-        <v>0</v>
-      </c>
-      <c r="O23" s="10">
-        <v>0</v>
-      </c>
-      <c r="P23" s="8">
-        <v>0</v>
-      </c>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10"/>
       <c r="Q23" s="10"/>
       <c r="R23" s="10"/>
       <c r="S23" s="10"/>
@@ -13615,9 +14167,15 @@
       <c r="P24" s="8">
         <v>0</v>
       </c>
-      <c r="Q24" s="6"/>
-      <c r="R24" s="6"/>
-      <c r="S24" s="6"/>
+      <c r="Q24" s="6">
+        <v>0</v>
+      </c>
+      <c r="R24" s="6">
+        <v>0</v>
+      </c>
+      <c r="S24" s="8">
+        <v>0</v>
+      </c>
       <c r="T24" s="6"/>
       <c r="U24" s="6"/>
       <c r="V24" s="6"/>
@@ -13686,9 +14244,15 @@
       <c r="P25" s="8">
         <v>62.5</v>
       </c>
-      <c r="Q25" s="10"/>
-      <c r="R25" s="10"/>
-      <c r="S25" s="10"/>
+      <c r="Q25" s="10">
+        <v>9</v>
+      </c>
+      <c r="R25" s="10">
+        <v>154</v>
+      </c>
+      <c r="S25" s="8">
+        <v>58.44</v>
+      </c>
       <c r="T25" s="10"/>
       <c r="U25" s="10"/>
       <c r="V25" s="10"/>
@@ -13757,9 +14321,15 @@
       <c r="P26" s="8">
         <v>0</v>
       </c>
-      <c r="Q26" s="6"/>
-      <c r="R26" s="6"/>
-      <c r="S26" s="6"/>
+      <c r="Q26" s="6">
+        <v>0</v>
+      </c>
+      <c r="R26" s="6">
+        <v>0</v>
+      </c>
+      <c r="S26" s="8">
+        <v>0</v>
+      </c>
       <c r="T26" s="6"/>
       <c r="U26" s="6"/>
       <c r="V26" s="6"/>
@@ -13828,9 +14398,15 @@
       <c r="P27" s="7">
         <v>17.73</v>
       </c>
-      <c r="Q27" s="10"/>
-      <c r="R27" s="10"/>
-      <c r="S27" s="10"/>
+      <c r="Q27" s="10">
+        <v>17</v>
+      </c>
+      <c r="R27" s="10">
+        <v>959</v>
+      </c>
+      <c r="S27" s="7">
+        <v>17.73</v>
+      </c>
       <c r="T27" s="10"/>
       <c r="U27" s="10"/>
       <c r="V27" s="10"/>
@@ -13899,9 +14475,15 @@
       <c r="P28" s="8">
         <v>0</v>
       </c>
-      <c r="Q28" s="6"/>
-      <c r="R28" s="6"/>
-      <c r="S28" s="6"/>
+      <c r="Q28" s="6">
+        <v>0</v>
+      </c>
+      <c r="R28" s="6">
+        <v>0</v>
+      </c>
+      <c r="S28" s="8">
+        <v>0</v>
+      </c>
       <c r="T28" s="6"/>
       <c r="U28" s="6"/>
       <c r="V28" s="6"/>
@@ -13970,9 +14552,15 @@
       <c r="P29" s="8">
         <v>0</v>
       </c>
-      <c r="Q29" s="10"/>
-      <c r="R29" s="10"/>
-      <c r="S29" s="10"/>
+      <c r="Q29" s="10">
+        <v>0</v>
+      </c>
+      <c r="R29" s="10">
+        <v>0</v>
+      </c>
+      <c r="S29" s="8">
+        <v>0</v>
+      </c>
       <c r="T29" s="10"/>
       <c r="U29" s="10"/>
       <c r="V29" s="10"/>
@@ -14041,9 +14629,15 @@
       <c r="P30" s="8">
         <v>0</v>
       </c>
-      <c r="Q30" s="6"/>
-      <c r="R30" s="6"/>
-      <c r="S30" s="6"/>
+      <c r="Q30" s="6">
+        <v>0</v>
+      </c>
+      <c r="R30" s="6">
+        <v>0</v>
+      </c>
+      <c r="S30" s="8">
+        <v>0</v>
+      </c>
       <c r="T30" s="6"/>
       <c r="U30" s="6"/>
       <c r="V30" s="6"/>
@@ -14112,9 +14706,15 @@
       <c r="P31" s="7">
         <v>20.32</v>
       </c>
-      <c r="Q31" s="11"/>
-      <c r="R31" s="11"/>
-      <c r="S31" s="11"/>
+      <c r="Q31" s="11">
+        <v>43</v>
+      </c>
+      <c r="R31" s="11">
+        <v>2166</v>
+      </c>
+      <c r="S31" s="7">
+        <v>19.85</v>
+      </c>
       <c r="T31" s="11"/>
       <c r="U31" s="11"/>
       <c r="V31" s="11"/>

</xml_diff>